<commit_message>
changes related to excel upload
</commit_message>
<xml_diff>
--- a/src/main/resources/Customer Registration Details.xlsx
+++ b/src/main/resources/Customer Registration Details.xlsx
@@ -1,11 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="11028"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81A30FBB-8D18-0F4D-9513-33AF30B86712}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="600" windowWidth="23400" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="600" windowWidth="20730" windowHeight="10425"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -17,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="28">
   <si>
     <t>S.No.</t>
   </si>
@@ -74,13 +73,40 @@
   </si>
   <si>
     <t>Ablock</t>
+  </si>
+  <si>
+    <t>vimal$#!</t>
+  </si>
+  <si>
+    <t>kvk9889gma</t>
+  </si>
+  <si>
+    <t>villa-9999</t>
+  </si>
+  <si>
+    <t>kvk</t>
+  </si>
+  <si>
+    <t>vimala</t>
+  </si>
+  <si>
+    <t>kumari</t>
+  </si>
+  <si>
+    <t>kv9889@gmail.com</t>
+  </si>
+  <si>
+    <t>k9889@gmail.com</t>
+  </si>
+  <si>
+    <t>kvk988@gmail.com</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -101,6 +127,34 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="6"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -127,7 +181,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -136,6 +190,18 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -157,9 +223,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -197,7 +263,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -231,7 +297,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -266,10 +331,9 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -442,23 +506,23 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I10"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:I11"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="7.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.28515625" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="22" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.33203125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="18.83203125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="18.33203125" style="1" customWidth="1"/>
-    <col min="6" max="6" width="18.5" style="1" customWidth="1"/>
-    <col min="7" max="7" width="19.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="37.5" style="1" customWidth="1"/>
+    <col min="3" max="3" width="16.28515625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="18.85546875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="18.28515625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="18.42578125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="19.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="37.42578125" style="1" customWidth="1"/>
     <col min="9" max="9" width="19" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="16384" width="9.1640625" style="1"/>
+    <col min="10" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9" s="2" customFormat="1" ht="27.75" customHeight="1">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -487,11 +551,11 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:9">
       <c r="A2" s="1">
         <v>1</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="5" t="s">
         <v>16</v>
       </c>
       <c r="C2" s="1" t="s">
@@ -516,14 +580,14 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:9">
       <c r="A3" s="1">
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" s="5" t="s">
         <v>17</v>
       </c>
       <c r="D3" s="1" t="s">
@@ -545,7 +609,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:9">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -555,6 +619,7 @@
       <c r="C4" s="1" t="s">
         <v>9</v>
       </c>
+      <c r="D4" s="5"/>
       <c r="E4" s="1" t="s">
         <v>11</v>
       </c>
@@ -571,7 +636,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:9">
       <c r="A5" s="1">
         <v>4</v>
       </c>
@@ -581,8 +646,8 @@
       <c r="C5" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="1" t="s">
-        <v>10</v>
+      <c r="D5" s="4" t="s">
+        <v>19</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>11</v>
@@ -600,7 +665,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:9">
       <c r="A6" s="1">
         <v>5</v>
       </c>
@@ -619,8 +684,8 @@
       <c r="F6" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="G6" s="1">
-        <v>8498890000</v>
+      <c r="G6" s="5">
+        <v>849889</v>
       </c>
       <c r="H6" s="3" t="s">
         <v>13</v>
@@ -629,7 +694,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:9">
       <c r="A7" s="1">
         <v>6</v>
       </c>
@@ -651,22 +716,22 @@
       <c r="G7" s="1">
         <v>8498890000</v>
       </c>
-      <c r="H7" s="3" t="s">
-        <v>13</v>
+      <c r="H7" s="4" t="s">
+        <v>20</v>
       </c>
       <c r="I7" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A8" s="1">
+    <row r="8" spans="1:9">
+      <c r="A8" s="7">
         <v>7</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B8" s="6" t="s">
         <v>15</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>10</v>
@@ -687,7 +752,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:9">
       <c r="A9" s="1">
         <v>8</v>
       </c>
@@ -698,25 +763,25 @@
         <v>9</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="F9" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="F9" s="5" t="s">
         <v>12</v>
       </c>
       <c r="G9" s="1">
-        <v>8498890000</v>
+        <v>8498890001</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="I9" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:9">
       <c r="A10" s="1">
         <v>9</v>
       </c>
@@ -726,10 +791,10 @@
       <c r="C10" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D10" s="1" t="s">
+      <c r="D10" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="E10" s="1" t="s">
+      <c r="E10" s="5" t="s">
         <v>11</v>
       </c>
       <c r="F10" s="1" t="s">
@@ -739,42 +804,84 @@
         <v>8498890000</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>13</v>
+        <v>26</v>
       </c>
       <c r="I10" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9">
+      <c r="A11" s="1">
+        <v>10</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G11" s="1">
+        <v>8498890002</v>
+      </c>
+      <c r="H11" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="I11" s="5" t="s">
         <v>14</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="H2" r:id="rId1" xr:uid="{8C45A32E-04D9-DA49-99FA-411BCCDDD89E}"/>
-    <hyperlink ref="H3" r:id="rId2" xr:uid="{B01B57CA-0CCD-C64E-AF5C-19D924AE350E}"/>
-    <hyperlink ref="H4" r:id="rId3" xr:uid="{F93EC6EB-60A9-2440-819D-8DE2F30C79FC}"/>
-    <hyperlink ref="H5" r:id="rId4" xr:uid="{3D447722-EE6A-8D47-BED9-835747EBFDA0}"/>
-    <hyperlink ref="H6" r:id="rId5" xr:uid="{9E870D59-8171-2841-BCB5-F9DD342A53AB}"/>
-    <hyperlink ref="H7" r:id="rId6" xr:uid="{2DA82C46-1069-5B45-B5FB-444E4CAFF60E}"/>
-    <hyperlink ref="H8" r:id="rId7" xr:uid="{E6919AA7-DED2-8D4E-A27F-2D12CA21222C}"/>
-    <hyperlink ref="H9" r:id="rId8" xr:uid="{6D527C75-0D43-C84A-997F-9F358FF1DBF7}"/>
-    <hyperlink ref="H10" r:id="rId9" xr:uid="{C0B885D9-909F-E246-BA1F-19908A964892}"/>
+    <hyperlink ref="H2" r:id="rId1"/>
+    <hyperlink ref="H3" r:id="rId2"/>
+    <hyperlink ref="H4" r:id="rId3"/>
+    <hyperlink ref="H5" r:id="rId4"/>
+    <hyperlink ref="H6" r:id="rId5"/>
+    <hyperlink ref="D5" r:id="rId6" display="vimal@#"/>
+    <hyperlink ref="H7" r:id="rId7" display="kvk9889@gma"/>
+    <hyperlink ref="H9" r:id="rId8"/>
+    <hyperlink ref="H10" r:id="rId9"/>
+    <hyperlink ref="H11" r:id="rId10"/>
+    <hyperlink ref="H8" r:id="rId11"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId10"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId12"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="7.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.28515625" customWidth="1"/>
+    <col min="4" max="4" width="18.85546875" customWidth="1"/>
+    <col min="5" max="5" width="18.28515625" customWidth="1"/>
+    <col min="6" max="6" width="18.42578125" customWidth="1"/>
+    <col min="7" max="7" width="19.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="37.42578125" customWidth="1"/>
+    <col min="9" max="9" width="19" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>